<commit_message>
Fix signature text overlap, date duplication, default department name in reports, and improve dynamic weekend styling
</commit_message>
<xml_diff>
--- a/Bao_cao_cham_cong_Thang_7_2026_TEST.xlsx
+++ b/Bao_cao_cham_cong_Thang_7_2026_TEST.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="704" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="117">
   <si>
     <r>
       <t xml:space="preserve">Đơn vị: </t>
@@ -262,127 +262,121 @@
     <t>Hải Vân, ngày 31 tháng 07 năm 2026</t>
   </si>
   <si>
+    <t>Bác sĩ Nguyễn Văn Trưởng</t>
+  </si>
+  <si>
+    <t>Ký hiệu chấm công:</t>
+  </si>
+  <si>
+    <t>Lương Thời gian</t>
+  </si>
+  <si>
+    <t>Hội nghị, học tập</t>
+  </si>
+  <si>
+    <t>Nghỉ ốm</t>
+  </si>
+  <si>
+    <t>Ô</t>
+  </si>
+  <si>
+    <t>Công tác</t>
+  </si>
+  <si>
+    <t>CT</t>
+  </si>
+  <si>
+    <t>Con ốm</t>
+  </si>
+  <si>
+    <t>Cô</t>
+  </si>
+  <si>
+    <t>Trực</t>
+  </si>
+  <si>
+    <t>Thai sản</t>
+  </si>
+  <si>
+    <t>Ts</t>
+  </si>
+  <si>
+    <t>Trực dịch</t>
+  </si>
+  <si>
+    <t>Td</t>
+  </si>
+  <si>
+    <t>Nghỉ không lương</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Chống dịch</t>
+  </si>
+  <si>
+    <t>cd</t>
+  </si>
+  <si>
+    <t>Nghỉ Phép</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Bù lễ</t>
+  </si>
+  <si>
+    <t>BL</t>
+  </si>
+  <si>
+    <t>Trực tiêm chủng</t>
+  </si>
+  <si>
+    <t>TTc</t>
+  </si>
+  <si>
+    <t>Phép chế độ</t>
+  </si>
+  <si>
+    <t>Pcđ</t>
+  </si>
+  <si>
+    <t>Tiêm chủng</t>
+  </si>
+  <si>
+    <t>Đơn vị: Trạm Y tế phường Hải Vân</t>
+  </si>
+  <si>
+    <t>BẢNG CHẤM CÔNG TRỰC</t>
+  </si>
+  <si>
+    <t>Tháng 07 Năm 2026</t>
+  </si>
+  <si>
+    <t>Mã đơn vị QHN:……………….</t>
+  </si>
+  <si>
+    <t>Tổng số ngày trong tháng</t>
+  </si>
+  <si>
+    <t>Ngày thường</t>
+  </si>
+  <si>
+    <t>Ngày thứ bảy, CN</t>
+  </si>
+  <si>
+    <t>Ngày Lễ</t>
+  </si>
+  <si>
+    <t>Tổng cộng</t>
+  </si>
+  <si>
+    <t>Tổng cộng: 5</t>
+  </si>
+  <si>
     <t xml:space="preserve">    Người chấm công</t>
-  </si>
-  <si>
-    <t>Phụ trách bộ phận</t>
-  </si>
-  <si>
-    <t>Trưởng khoa</t>
-  </si>
-  <si>
-    <t>Bác sĩ Nguyễn Văn Trưởng</t>
-  </si>
-  <si>
-    <t>Ký hiệu chấm công:</t>
-  </si>
-  <si>
-    <t>Lương Thời gian</t>
-  </si>
-  <si>
-    <t>Hội nghị, học tập</t>
-  </si>
-  <si>
-    <t>Nghỉ ốm</t>
-  </si>
-  <si>
-    <t>Ô</t>
-  </si>
-  <si>
-    <t>Công tác</t>
-  </si>
-  <si>
-    <t>CT</t>
-  </si>
-  <si>
-    <t>Con ốm</t>
-  </si>
-  <si>
-    <t>Cô</t>
-  </si>
-  <si>
-    <t>Trực</t>
-  </si>
-  <si>
-    <t>Thai sản</t>
-  </si>
-  <si>
-    <t>Ts</t>
-  </si>
-  <si>
-    <t>Trực dịch</t>
-  </si>
-  <si>
-    <t>Td</t>
-  </si>
-  <si>
-    <t>Nghỉ không lương</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Chống dịch</t>
-  </si>
-  <si>
-    <t>cd</t>
-  </si>
-  <si>
-    <t>Nghỉ Phép</t>
-  </si>
-  <si>
-    <t>P</t>
-  </si>
-  <si>
-    <t>Bù lễ</t>
-  </si>
-  <si>
-    <t>BL</t>
-  </si>
-  <si>
-    <t>Trực tiêm chủng</t>
-  </si>
-  <si>
-    <t>TTc</t>
-  </si>
-  <si>
-    <t>Phép chế độ</t>
-  </si>
-  <si>
-    <t>Pcđ</t>
-  </si>
-  <si>
-    <t>Tiêm chủng</t>
-  </si>
-  <si>
-    <t>Đơn vị: Trạm Y tế phường Hải Vân</t>
-  </si>
-  <si>
-    <t>BẢNG CHẤM CÔNG TRỰC</t>
-  </si>
-  <si>
-    <t>Tháng 07 Năm 2026</t>
-  </si>
-  <si>
-    <t>Mã đơn vị QHN:……………….</t>
-  </si>
-  <si>
-    <t>Tổng số ngày trong tháng</t>
-  </si>
-  <si>
-    <t>Ngày thường</t>
-  </si>
-  <si>
-    <t>Ngày thứ bảy, CN</t>
-  </si>
-  <si>
-    <t>Ngày Lễ</t>
-  </si>
-  <si>
-    <t>Tổng cộng</t>
-  </si>
-  <si>
-    <t>Tổng cộng: 5</t>
   </si>
   <si>
     <t>24h</t>
@@ -606,8 +600,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFE2E2E2"/>
       </patternFill>
     </fill>
   </fills>
@@ -3396,13 +3389,27 @@
       <c r="Q16" s="8"/>
       <c r="R16" s="8"/>
       <c r="S16" s="8"/>
-      <c r="T16" s="8"/>
-      <c r="U16" s="8"/>
-      <c r="V16" s="8"/>
-      <c r="W16" s="8"/>
-      <c r="X16" s="8"/>
-      <c r="Y16" s="8"/>
-      <c r="Z16" s="8"/>
+      <c r="T16" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="U16" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="V16" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="W16" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="X16" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y16" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z16" s="8" t="s">
+        <v>51</v>
+      </c>
       <c r="AA16" s="30" t="s">
         <v>63</v>
       </c>
@@ -3421,7 +3428,7 @@
     </row>
     <row r="17" ht="15.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A17" s="31" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="B17" s="31"/>
       <c r="C17" s="3"/>
@@ -3434,7 +3441,7 @@
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
       <c r="L17" s="31" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="M17" s="31"/>
       <c r="N17" s="31"/>
@@ -3451,7 +3458,7 @@
       <c r="Y17" s="1"/>
       <c r="Z17" s="1"/>
       <c r="AA17" s="31" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="AB17" s="31"/>
       <c r="AC17" s="31"/>
@@ -3475,14 +3482,14 @@
         <v>58</v>
       </c>
       <c r="AA21" s="32" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="33" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D22" s="33"/>
       <c r="E22" s="33"/>
@@ -3525,7 +3532,7 @@
       <c r="A23" s="35"/>
       <c r="B23" s="36"/>
       <c r="C23" s="37" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D23" s="37"/>
       <c r="E23" s="37"/>
@@ -3548,7 +3555,7 @@
       <c r="T23" s="39"/>
       <c r="U23" s="39"/>
       <c r="V23" s="39" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="W23" s="39"/>
       <c r="X23" s="39"/>
@@ -3574,7 +3581,7 @@
       <c r="A24" s="41"/>
       <c r="B24" s="39"/>
       <c r="C24" s="42" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D24" s="42"/>
       <c r="E24" s="42"/>
@@ -3584,7 +3591,7 @@
       <c r="I24" s="37"/>
       <c r="J24" s="37"/>
       <c r="K24" s="38" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="L24" s="38"/>
       <c r="M24" s="39"/>
@@ -3597,7 +3604,7 @@
       <c r="T24" s="39"/>
       <c r="U24" s="39"/>
       <c r="V24" s="39" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="W24" s="39"/>
       <c r="X24" s="39"/>
@@ -3605,7 +3612,7 @@
       <c r="Z24" s="39"/>
       <c r="AA24" s="39"/>
       <c r="AB24" s="39" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="AC24" s="39"/>
       <c r="AD24" s="39"/>
@@ -3623,7 +3630,7 @@
       <c r="A25" s="41"/>
       <c r="B25" s="39"/>
       <c r="C25" s="37" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D25" s="37"/>
       <c r="E25" s="37"/>
@@ -3633,7 +3640,7 @@
       <c r="I25" s="37"/>
       <c r="J25" s="37"/>
       <c r="K25" s="38" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="L25" s="38"/>
       <c r="M25" s="39"/>
@@ -3646,7 +3653,7 @@
       <c r="T25" s="39"/>
       <c r="U25" s="39"/>
       <c r="V25" s="39" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="W25" s="39"/>
       <c r="X25" s="39"/>
@@ -3672,7 +3679,7 @@
       <c r="A26" s="41"/>
       <c r="B26" s="39"/>
       <c r="C26" s="37" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D26" s="37"/>
       <c r="E26" s="37"/>
@@ -3682,7 +3689,7 @@
       <c r="I26" s="37"/>
       <c r="J26" s="37"/>
       <c r="K26" s="38" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="L26" s="38"/>
       <c r="M26" s="39"/>
@@ -3721,7 +3728,7 @@
       <c r="A27" s="41"/>
       <c r="B27" s="39"/>
       <c r="C27" s="37" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D27" s="37"/>
       <c r="E27" s="37"/>
@@ -3731,7 +3738,7 @@
       <c r="I27" s="37"/>
       <c r="J27" s="37"/>
       <c r="K27" s="38" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="L27" s="38"/>
       <c r="M27" s="39"/>
@@ -3744,7 +3751,7 @@
       <c r="T27" s="39"/>
       <c r="U27" s="39"/>
       <c r="V27" s="39" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="W27" s="39"/>
       <c r="X27" s="39"/>
@@ -3752,7 +3759,7 @@
       <c r="Z27" s="39"/>
       <c r="AA27" s="39"/>
       <c r="AB27" s="38" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="AC27" s="38"/>
       <c r="AD27" s="39"/>
@@ -3770,7 +3777,7 @@
       <c r="A28" s="44"/>
       <c r="B28" s="38"/>
       <c r="C28" s="42" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D28" s="42"/>
       <c r="E28" s="42"/>
@@ -3780,7 +3787,7 @@
       <c r="I28" s="42"/>
       <c r="J28" s="42"/>
       <c r="K28" s="38" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="L28" s="38"/>
       <c r="M28" s="38"/>
@@ -3793,7 +3800,7 @@
       <c r="T28" s="38"/>
       <c r="U28" s="38"/>
       <c r="V28" s="39" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="W28" s="39"/>
       <c r="X28" s="39"/>
@@ -3801,7 +3808,7 @@
       <c r="Z28" s="39"/>
       <c r="AA28" s="39"/>
       <c r="AB28" s="38" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="AC28" s="38"/>
       <c r="AD28" s="39"/>
@@ -3818,7 +3825,7 @@
     <row r="29" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A29" s="41"/>
       <c r="C29" s="39" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D29" s="39"/>
       <c r="E29" s="39"/>
@@ -3828,7 +3835,7 @@
       <c r="I29" s="37"/>
       <c r="J29" s="37"/>
       <c r="K29" s="37" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L29" s="39"/>
       <c r="M29" s="39"/>
@@ -3841,7 +3848,7 @@
       <c r="T29" s="39"/>
       <c r="U29" s="39"/>
       <c r="V29" s="39" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="W29" s="39"/>
       <c r="X29" s="39"/>
@@ -3849,7 +3856,7 @@
       <c r="Z29" s="39"/>
       <c r="AA29" s="39"/>
       <c r="AB29" s="39" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="AC29" s="39"/>
       <c r="AD29" s="41"/>
@@ -3860,13 +3867,13 @@
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.25">
       <c r="C30" s="39" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="K30" s="39" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="V30" s="39" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="W30" s="39"/>
       <c r="X30" s="39"/>
@@ -3932,7 +3939,7 @@
   <sheetData>
     <row r="1" ht="18.75" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A1" s="48" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B1" s="48"/>
       <c r="C1" s="48"/>
@@ -3942,7 +3949,7 @@
       <c r="G1" s="48"/>
       <c r="H1" s="48"/>
       <c r="I1" s="49" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="J1" s="49"/>
       <c r="K1" s="49"/>
@@ -3985,7 +3992,7 @@
       <c r="G2" s="50"/>
       <c r="H2" s="50"/>
       <c r="I2" s="51" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="J2" s="51"/>
       <c r="K2" s="51"/>
@@ -4018,7 +4025,7 @@
     </row>
     <row r="3" ht="19.5" customHeight="1" spans="1:37" s="52" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="53" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B3" s="53"/>
       <c r="C3" s="53"/>
@@ -4137,7 +4144,7 @@
       <c r="AF5" s="14"/>
       <c r="AG5" s="15"/>
       <c r="AH5" s="13" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="AI5" s="14"/>
       <c r="AJ5" s="14"/>
@@ -4240,16 +4247,16 @@
         <v>42</v>
       </c>
       <c r="AH6" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="AI6" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="AJ6" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="AK6" s="19" t="s">
         <v>100</v>
-      </c>
-      <c r="AI6" s="18" t="s">
-        <v>101</v>
-      </c>
-      <c r="AJ6" s="19" t="s">
-        <v>102</v>
-      </c>
-      <c r="AK6" s="19" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="7" ht="20.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
@@ -4808,7 +4815,7 @@
     <row r="12" ht="20.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A12" s="28"/>
       <c r="B12" s="29" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C12" s="28"/>
       <c r="D12" s="28"/>
@@ -4874,15 +4881,33 @@
       <c r="Q13" s="58"/>
       <c r="R13" s="58"/>
       <c r="S13" s="58"/>
-      <c r="T13" s="58"/>
-      <c r="U13" s="58"/>
-      <c r="V13" s="58"/>
-      <c r="W13" s="58"/>
-      <c r="X13" s="58"/>
-      <c r="Y13" s="58"/>
-      <c r="Z13" s="58"/>
-      <c r="AA13" s="58"/>
-      <c r="AB13" s="58"/>
+      <c r="T13" s="58" t="s">
+        <v>51</v>
+      </c>
+      <c r="U13" s="58" t="s">
+        <v>51</v>
+      </c>
+      <c r="V13" s="58" t="s">
+        <v>51</v>
+      </c>
+      <c r="W13" s="58" t="s">
+        <v>51</v>
+      </c>
+      <c r="X13" s="58" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y13" s="58" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z13" s="58" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA13" s="58" t="s">
+        <v>51</v>
+      </c>
+      <c r="AB13" s="58" t="s">
+        <v>51</v>
+      </c>
       <c r="AC13" s="59" t="s">
         <v>63</v>
       </c>
@@ -4898,7 +4923,7 @@
     <row r="14" ht="15.75" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A14" s="60"/>
       <c r="B14" s="50" t="s">
-        <v>64</v>
+        <v>102</v>
       </c>
       <c r="C14" s="61"/>
       <c r="D14" s="61"/>
@@ -4910,7 +4935,7 @@
       <c r="J14" s="61"/>
       <c r="K14" s="61"/>
       <c r="L14" s="51" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="M14" s="51"/>
       <c r="N14" s="51"/>
@@ -4927,7 +4952,7 @@
       <c r="Y14" s="61"/>
       <c r="Z14" s="61"/>
       <c r="AA14" s="62" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="AB14" s="62"/>
       <c r="AC14" s="62"/>
@@ -4948,7 +4973,7 @@
         <v>58</v>
       </c>
       <c r="AA18" s="32" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:37" x14ac:dyDescent="0.25">
@@ -4994,7 +5019,7 @@
       <c r="A20" s="61"/>
       <c r="B20" s="61"/>
       <c r="C20" s="64" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D20" s="64"/>
       <c r="E20" s="64"/>
@@ -5035,11 +5060,11 @@
       <c r="A21" s="46"/>
       <c r="B21" s="46"/>
       <c r="C21" s="46" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D21" s="46"/>
       <c r="E21" s="46" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F21" s="46"/>
       <c r="G21" s="46"/>
@@ -5080,7 +5105,7 @@
       <c r="A22" s="46"/>
       <c r="B22" s="46"/>
       <c r="C22" s="46" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D22" s="46"/>
       <c r="E22" s="46"/>
@@ -5090,7 +5115,7 @@
       <c r="I22" s="46"/>
       <c r="J22" s="46"/>
       <c r="K22" s="64" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="L22" s="64"/>
       <c r="M22" s="46"/>
@@ -5123,7 +5148,7 @@
       <c r="A23" s="67"/>
       <c r="B23" s="67"/>
       <c r="C23" s="55" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D23" s="46"/>
       <c r="E23" s="46"/>
@@ -5166,7 +5191,7 @@
       <c r="A24" s="46"/>
       <c r="B24" s="68"/>
       <c r="C24" s="64" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D24" s="46"/>
       <c r="E24" s="64"/>
@@ -5176,7 +5201,7 @@
       <c r="I24" s="64"/>
       <c r="J24" s="46"/>
       <c r="K24" s="64" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -5205,7 +5230,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AH19"/>
+  <dimension ref="A1:AI19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="26.5703125" customWidth="1"/>
@@ -5215,7 +5240,7 @@
   <sheetData>
     <row r="1" ht="18.75" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5223,7 +5248,7 @@
       <c r="E1" s="69"/>
       <c r="F1" s="70"/>
       <c r="G1" s="71" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H1" s="71"/>
       <c r="I1" s="71"/>
@@ -5262,7 +5287,7 @@
       <c r="E2" s="72"/>
       <c r="F2" s="72"/>
       <c r="G2" s="73" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H2" s="73"/>
       <c r="I2" s="73"/>
@@ -5407,7 +5432,7 @@
       <c r="AF5" s="77"/>
       <c r="AG5" s="78"/>
       <c r="AH5" s="79" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" ht="29.25" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
@@ -5615,7 +5640,7 @@
     <row r="8" ht="22.5" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A8" s="84"/>
       <c r="B8" s="85" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C8" s="85"/>
       <c r="D8" s="85"/>
@@ -5652,7 +5677,7 @@
         <f>SUM(AH7:AH7)</f>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1" spans="1:34" s="86" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" ht="15.75" customHeight="1" spans="1:35" s="86" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="87"/>
       <c r="B9" s="87"/>
       <c r="C9" s="87"/>
@@ -5672,10 +5697,21 @@
       <c r="Q9" s="88"/>
       <c r="R9" s="88"/>
       <c r="S9" s="88"/>
-      <c r="T9" s="88"/>
-      <c r="U9" s="88"/>
-      <c r="W9" s="89"/>
-      <c r="X9" s="89"/>
+      <c r="T9" s="88" t="s">
+        <v>51</v>
+      </c>
+      <c r="U9" s="88" t="s">
+        <v>51</v>
+      </c>
+      <c r="V9" s="86" t="s">
+        <v>51</v>
+      </c>
+      <c r="W9" s="89" t="s">
+        <v>51</v>
+      </c>
+      <c r="X9" s="89" t="s">
+        <v>51</v>
+      </c>
       <c r="Y9" s="90" t="s">
         <v>63</v>
       </c>
@@ -5688,11 +5724,14 @@
       <c r="AF9" s="90"/>
       <c r="AG9" s="90"/>
       <c r="AH9" s="90"/>
+      <c r="AI9" s="86" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="10" ht="15.75" customHeight="1" spans="1:34" s="86" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="91"/>
       <c r="B10" s="92" t="s">
-        <v>64</v>
+        <v>102</v>
       </c>
       <c r="C10" s="91"/>
       <c r="D10" s="93"/>
@@ -5704,7 +5743,7 @@
       <c r="J10" s="93"/>
       <c r="K10" s="93"/>
       <c r="L10" s="94" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="M10" s="94"/>
       <c r="N10" s="94"/>
@@ -5719,7 +5758,7 @@
       <c r="W10" s="86"/>
       <c r="X10" s="91"/>
       <c r="Y10" s="95" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="Z10" s="95"/>
       <c r="AA10" s="95"/>
@@ -5742,7 +5781,7 @@
         <v>58</v>
       </c>
       <c r="Y14" s="32" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
@@ -5785,7 +5824,7 @@
       <c r="A16" s="1"/>
       <c r="B16" s="97"/>
       <c r="C16" s="98" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D16" s="98"/>
       <c r="E16" s="98"/>
@@ -5823,7 +5862,7 @@
       <c r="A17" s="1"/>
       <c r="B17" s="99"/>
       <c r="C17" s="41" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D17" s="100"/>
       <c r="E17" s="100"/>
@@ -5863,7 +5902,7 @@
       <c r="A18" s="41"/>
       <c r="B18" s="69"/>
       <c r="C18" s="41" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D18" s="100"/>
       <c r="E18" s="100"/>
@@ -5873,7 +5912,7 @@
       <c r="I18" s="102"/>
       <c r="J18" s="102"/>
       <c r="K18" s="103" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="L18" s="103"/>
       <c r="M18" s="100"/>
@@ -5903,7 +5942,7 @@
       <c r="A19" s="41"/>
       <c r="B19" s="69"/>
       <c r="C19" s="41" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D19" s="100"/>
       <c r="E19" s="100"/>
@@ -5966,7 +6005,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AH20"/>
+  <dimension ref="A1:AI20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24.85546875" customWidth="1"/>
@@ -5976,7 +6015,7 @@
   <sheetData>
     <row r="1" ht="18.75" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A1" s="48" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B1" s="48"/>
       <c r="C1" s="48"/>
@@ -5984,7 +6023,7 @@
       <c r="E1" s="48"/>
       <c r="F1" s="48"/>
       <c r="G1" s="71" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H1" s="71"/>
       <c r="I1" s="71"/>
@@ -6024,7 +6063,7 @@
       <c r="E2" s="48"/>
       <c r="F2" s="48"/>
       <c r="G2" s="73" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H2" s="73"/>
       <c r="I2" s="73"/>
@@ -6169,7 +6208,7 @@
       <c r="AF5" s="106"/>
       <c r="AG5" s="107"/>
       <c r="AH5" s="79" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
@@ -6273,7 +6312,7 @@
     <row r="7" ht="22.5" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A7" s="75"/>
       <c r="B7" s="108" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C7" s="23" t="s">
         <v>12</v>
@@ -6477,7 +6516,7 @@
     <row r="9" ht="22.5" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A9" s="84"/>
       <c r="B9" s="85" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C9" s="85"/>
       <c r="D9" s="85"/>
@@ -6514,7 +6553,7 @@
         <f>SUM(AH8:AH8)</f>
       </c>
     </row>
-    <row r="10" ht="15.75" customHeight="1" spans="1:34" s="86" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" ht="15.75" customHeight="1" spans="1:35" s="86" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="87"/>
       <c r="B10" s="87"/>
       <c r="C10" s="87"/>
@@ -6534,10 +6573,21 @@
       <c r="Q10" s="88"/>
       <c r="R10" s="88"/>
       <c r="S10" s="88"/>
-      <c r="T10" s="88"/>
-      <c r="U10" s="88"/>
-      <c r="W10" s="89"/>
-      <c r="X10" s="89"/>
+      <c r="T10" s="88" t="s">
+        <v>51</v>
+      </c>
+      <c r="U10" s="88" t="s">
+        <v>51</v>
+      </c>
+      <c r="V10" s="86" t="s">
+        <v>51</v>
+      </c>
+      <c r="W10" s="89" t="s">
+        <v>51</v>
+      </c>
+      <c r="X10" s="89" t="s">
+        <v>51</v>
+      </c>
       <c r="Y10" s="90" t="s">
         <v>63</v>
       </c>
@@ -6550,11 +6600,14 @@
       <c r="AF10" s="90"/>
       <c r="AG10" s="90"/>
       <c r="AH10" s="90"/>
+      <c r="AI10" s="86" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="11" ht="15.75" customHeight="1" spans="1:34" s="86" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="91"/>
       <c r="B11" s="92" t="s">
-        <v>64</v>
+        <v>102</v>
       </c>
       <c r="C11" s="91"/>
       <c r="D11" s="93"/>
@@ -6566,7 +6619,7 @@
       <c r="J11" s="93"/>
       <c r="K11" s="93"/>
       <c r="L11" s="94" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="M11" s="94"/>
       <c r="N11" s="94"/>
@@ -6581,7 +6634,7 @@
       <c r="W11" s="86"/>
       <c r="X11" s="91"/>
       <c r="Y11" s="95" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="Z11" s="95"/>
       <c r="AA11" s="95"/>
@@ -6604,7 +6657,7 @@
         <v>58</v>
       </c>
       <c r="Y15" s="32" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">

</xml_diff>